<commit_message>
Actualización automática 2026-01-08 16:30:10
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>155.52</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>0 de 23</t>
+          <t>1 de 23</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2371,7 +2371,7 @@
         <v>5296.63</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>155.52</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>6000</v>
@@ -2712,7 +2712,7 @@
         <v>59467.53</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>912.4</v>
+        <v>1067.92</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-02-05 11:30:13
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>1222.04</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>0 de 23</t>
+          <t>1 de 23</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2290,7 +2290,7 @@
         <v>3632.07</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>1222.04</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>5000</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0</v>
+        <v>1222.04</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2735,9 +2735,9 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>1222.04</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>32950</v>
+        <v>31727.96</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.03708770864946889</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>1222.04</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40843.95</v>
+        <v>39621.91</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0</v>
+        <v>0.02991973107400239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-05 13:30:13
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1845,7 +1845,7 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>0</v>
+        <v>-658.35</v>
       </c>
       <c r="I23" s="2" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>940.5</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>0</v>
+        <v>-658.35</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>0</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>1222.04</v>
+        <v>563.6899999999999</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2883,13 +2883,13 @@
         <v>2350</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0</v>
+        <v>-658.35</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2350</v>
+        <v>3008.35</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>0</v>
+        <v>-0.2801489361702128</v>
       </c>
     </row>
     <row r="7">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>1222.04</v>
+        <v>563.6899999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>39621.91</v>
+        <v>40280.26</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.02991973107400239</v>
+        <v>0.01380106478438055</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-10 14:30:20
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>1115.22</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I17" s="2" t="n">
         <v>0</v>
@@ -1500,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>1280.37</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1966,32 +1966,32 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
+          <t>1 de 23</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>1 de 23</t>
+          <t>3 de 23</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2236,7 +2236,7 @@
         <v>3543.89</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>1115.22</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -2506,7 +2506,7 @@
         <v>3539.95</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0</v>
+        <v>2062.47</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>1500</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>-328.44</v>
+        <v>2849.25</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2883,13 +2883,13 @@
         <v>2350</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>-1504.8</v>
+        <v>-722.7</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>3854.8</v>
+        <v>3072.7</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.6403404255319148</v>
+        <v>-0.307531914893617</v>
       </c>
     </row>
     <row r="7">
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1222.04</v>
+        <v>3617.63</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>31727.96</v>
+        <v>29332.37</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.03708770864946889</v>
+        <v>0.109791502276176</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>-328.4400000000001</v>
+        <v>2849.25</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>41172.39</v>
+        <v>37994.7</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>-0.008041337823594437</v>
+        <v>0.06975941357287921</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-12 08:30:20
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1389,7 +1389,7 @@
         <v>0</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>0</v>
+        <v>2.12</v>
       </c>
       <c r="Q15" s="2" t="n">
         <v>0</v>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>3 de 23</t>
+          <t>4 de 23</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="P25" s="4" t="inlineStr">
         <is>
-          <t>0 de 23</t>
+          <t>1 de 23</t>
         </is>
       </c>
       <c r="Q25" s="4" t="inlineStr">
@@ -2452,7 +2452,7 @@
         <v>5818.17</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6500</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>3977.85</v>
+        <v>3986.22</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2931,13 +2931,13 @@
         <v>250</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>2.12</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>250</v>
+        <v>247.88</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>0.00848</v>
       </c>
     </row>
     <row r="9">
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>3617.63</v>
+        <v>3623.88</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>29332.37</v>
+        <v>29326.12</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.109791502276176</v>
+        <v>0.1099811836115326</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>3977.85</v>
+        <v>3986.22</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>36866.10000000001</v>
+        <v>36857.73</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.09739141292651664</v>
+        <v>0.09759633923751253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-18 08:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>1222.04</v>
+        <v>1202.95</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -2290,7 +2290,7 @@
         <v>3632.07</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1222.04</v>
+        <v>1202.95</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>5000</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>5891.089999999999</v>
+        <v>5872</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4746.65</v>
+        <v>4727.56</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>28203.35</v>
+        <v>28222.44</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1440561456752655</v>
+        <v>0.1434767830045524</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5891.089999999999</v>
+        <v>5872</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>34952.86</v>
+        <v>34971.95</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1442340909730817</v>
+        <v>0.1437667022900576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-19 15:30:22
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>6.25</v>
+        <v>2526.71</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -2452,7 +2452,7 @@
         <v>5818.17</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>8.369999999999999</v>
+        <v>2528.83</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6500</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>5872</v>
+        <v>8392.459999999999</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4727.56</v>
+        <v>7248.02</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>28222.44</v>
+        <v>25701.98</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1434767830045524</v>
+        <v>0.2199702579666161</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>5872</v>
+        <v>8392.460000000001</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>34971.95</v>
+        <v>32451.49</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1437667022900576</v>
+        <v>0.2054762088387631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-19 17:30:23
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>2526.71</v>
+        <v>1896.59</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -2452,7 +2452,7 @@
         <v>5818.17</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>2528.83</v>
+        <v>1898.71</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6500</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>8392.459999999999</v>
+        <v>7762.34</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2735,7 +2735,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>7248.02</v>
+        <v>6617.9</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>25701.98</v>
+        <v>26332.1</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2199702579666161</v>
+        <v>0.2008467374810319</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>8392.460000000001</v>
+        <v>7762.339999999999</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>32451.49</v>
+        <v>33081.61</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2054762088387631</v>
+        <v>0.1900487097844356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-02-23 14:30:22
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1115.22</v>
+        <v>2875.17</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1353,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>457.92</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -1380,7 +1380,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>1896.59</v>
+        <v>6538.96</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>0 de 23</t>
+          <t>1 de 23</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2236,7 +2236,7 @@
         <v>3543.89</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>1115.22</v>
+        <v>2875.17</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -2452,7 +2452,7 @@
         <v>5818.17</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1898.71</v>
+        <v>6999</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6500</v>
@@ -2712,7 +2712,7 @@
         <v>54049.74</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>7694.69</v>
+        <v>14554.93</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2735,7 +2735,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2811,13 +2811,13 @@
         <v>2183</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>457.92</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2183</v>
+        <v>1725.08</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>0.2097663765460376</v>
       </c>
     </row>
     <row r="4">
@@ -3051,13 +3051,13 @@
         <v>32950</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6617.9</v>
+        <v>13020.22</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>26332.1</v>
+        <v>19929.78</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2008467374810319</v>
+        <v>0.3951508345978755</v>
       </c>
     </row>
     <row r="14">
@@ -3118,13 +3118,13 @@
         <v>40843.95</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>7694.69</v>
+        <v>14554.93</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>33149.26</v>
+        <v>26289.02</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1883924057296123</v>
+        <v>0.3563546131067146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-05 12:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>1176.46</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>0 de 23</t>
+          <t>1 de 23</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2039,7 +2039,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2371,7 +2371,7 @@
         <v>1894.07</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>1176.46</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>6000</v>
@@ -2712,7 +2712,7 @@
         <v>15326.68</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>0</v>
+        <v>1176.46</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2735,9 +2735,9 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3051,13 +3051,13 @@
         <v>52623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>1176.46</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>52623</v>
+        <v>51446.54</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>0.02235638409060677</v>
       </c>
     </row>
     <row r="14">
@@ -3094,13 +3094,13 @@
         <v>57256.2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>1176.46</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>57256.2</v>
+        <v>56079.74000000001</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>0.02054729444147533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-10 12:30:24
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>1591.57</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1353,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>2719.84</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -1377,10 +1377,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>0</v>
+        <v>2869.45</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>2315.25</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1946,52 +1946,52 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
+          <t>1 de 23</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>0 de 23</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>0 de 23</t>
+          <t>1 de 23</t>
         </is>
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>1 de 23</t>
+          <t>3 de 23</t>
         </is>
       </c>
       <c r="N25" s="4" t="inlineStr">
@@ -2236,7 +2236,7 @@
         <v>2875.17</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>1591.57</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -2452,7 +2452,7 @@
         <v>7770.75</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>7904.54</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6500</v>
@@ -2712,7 +2712,7 @@
         <v>15326.68</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>1176.46</v>
+        <v>10672.57</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49000</v>
@@ -2736,7 +2736,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -2811,13 +2811,13 @@
         <v>2183</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0</v>
+        <v>2719.84</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2183</v>
+        <v>-536.8400000000001</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>1.245918460833715</v>
       </c>
     </row>
     <row r="4">
@@ -3027,13 +3027,13 @@
         <v>467</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>2869.45</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>467</v>
+        <v>-2402.45</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>6.144432548179871</v>
       </c>
     </row>
     <row r="13">
@@ -3051,13 +3051,13 @@
         <v>52623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1176.46</v>
+        <v>5083.28</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>51446.54</v>
+        <v>47539.72</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.02235638409060677</v>
+        <v>0.09659806548467399</v>
       </c>
     </row>
     <row r="14">
@@ -3094,13 +3094,13 @@
         <v>57256.2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1176.46</v>
+        <v>10672.57</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>56079.74000000001</v>
+        <v>46583.63</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.02054729444147533</v>
+        <v>0.1864002501039189</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-10 15:30:27
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MATERIALES DE CONSTRUCCION SUPERMACONSVI S.A.</t>
+          <t>MARIN DELGADO BRENDA MARIA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MEGAMAFERS S.A.</t>
+          <t>MATERIALES DE CONSTRUCCION SUPERMACONSVI S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1346,14 +1346,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MUÑOZ LOZA ROMMEL SEBASTIAN</t>
+          <t>MEGAMAFERS S.A.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2719.84</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>0</v>
@@ -1377,10 +1377,10 @@
         <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>2869.45</v>
+        <v>0</v>
       </c>
       <c r="M15" s="2" t="n">
-        <v>2315.25</v>
+        <v>0</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
@@ -1406,14 +1406,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORTEGA PAREDES RUDHT ELENA</t>
+          <t>MUÑOZ LOZA ROMMEL SEBASTIAN</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>2719.84</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>0</v>
@@ -1437,10 +1437,10 @@
         <v>0</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>0</v>
+        <v>2869.45</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>2315.25</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OÑATE PEREZ MERCY YOLANDA</t>
+          <t>ORTEGA PAREDES RUDHT ELENA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PADILLA MIER BERTHA MARIETA</t>
+          <t>OÑATE PEREZ MERCY YOLANDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAVIMARSA S.A.</t>
+          <t>PADILLA MIER BERTHA MARIETA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>REA ARMAS CARLOS FERNANDO</t>
+          <t>PAVIMARSA S.A.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SARZOSA UNDA JOSE DOMINGO</t>
+          <t>REA ARMAS CARLOS FERNANDO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SIGCHOS MORA FRANKLIN PORFIRIO</t>
+          <t>SARZOSA UNDA JOSE DOMINGO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TRUJILLO TORRES VINICIO RUBEN</t>
+          <t>SIGCHOS MORA FRANKLIN PORFIRIO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1886,137 +1886,197 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>TRUJILLO TORRES VINICIO RUBEN</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>TULCAN NARVAEZ EDITH MARITZA</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>1 de 23</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>1 de 23</t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="inlineStr">
-        <is>
-          <t>3 de 23</t>
-        </is>
-      </c>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="O25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="P25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="Q25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
-        </is>
-      </c>
-      <c r="R25" s="4" t="inlineStr">
-        <is>
-          <t>0 de 23</t>
+      <c r="C25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>1 de 24</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>1 de 24</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>3 de 24</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -2385,7 +2445,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MATERIALES DE CONSTRUCCION SUPERMACONSVI S.A.</t>
+          <t>MARIN DELGADO BRENDA MARIA</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -2412,23 +2472,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MEGAMAFERS S.A.</t>
+          <t>MATERIALES DE CONSTRUCCION SUPERMACONSVI S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>6009.13</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>10228.49</v>
+        <v>0</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>1128.6</v>
+        <v>0</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>6500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2439,20 +2499,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MUÑOZ LOZA ROMMEL SEBASTIAN</t>
+          <t>MEGAMAFERS S.A.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2701.41</v>
+        <v>6009.13</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>5818.17</v>
+        <v>10228.49</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>7770.75</v>
+        <v>1128.6</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>7904.54</v>
+        <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6500</v>
@@ -2466,23 +2526,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORTEGA PAREDES RUDHT ELENA</t>
+          <t>MUÑOZ LOZA ROMMEL SEBASTIAN</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0</v>
+        <v>2701.41</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>5818.17</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>7770.75</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>7904.54</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="17">
@@ -2493,23 +2553,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OÑATE PEREZ MERCY YOLANDA</t>
+          <t>ORTEGA PAREDES RUDHT ELENA</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>3091.73</v>
+        <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>3539.95</v>
+        <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1994.82</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -2520,23 +2580,23 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PADILLA MIER BERTHA MARIETA</t>
+          <t>OÑATE PEREZ MERCY YOLANDA</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>675.3200000000001</v>
+        <v>3091.73</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>6802.16</v>
+        <v>3539.95</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0</v>
+        <v>1994.82</v>
       </c>
       <c r="F18" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>5000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="19">
@@ -2547,14 +2607,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PAVIMARSA S.A.</t>
+          <t>PADILLA MIER BERTHA MARIETA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>0</v>
+        <v>675.3200000000001</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>6802.16</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -2563,7 +2623,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="20">
@@ -2574,7 +2634,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>REA ARMAS CARLOS FERNANDO</t>
+          <t>PAVIMARSA S.A.</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -2601,14 +2661,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SARZOSA UNDA JOSE DOMINGO</t>
+          <t>REA ARMAS CARLOS FERNANDO</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>-496.35</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>4415.8</v>
+        <v>0</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -2628,14 +2688,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SIGCHOS MORA FRANKLIN PORFIRIO</t>
+          <t>SARZOSA UNDA JOSE DOMINGO</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>0</v>
+        <v>-496.35</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>4415.8</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
@@ -2655,17 +2715,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>TRUJILLO TORRES VINICIO RUBEN</t>
+          <t>SIGCHOS MORA FRANKLIN PORFIRIO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1351.47</v>
+        <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>940.5</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>-1494</v>
+        <v>0</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0</v>
@@ -2682,39 +2742,66 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>TRUJILLO TORRES VINICIO RUBEN</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>1351.47</v>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>940.5</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>-1494</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>TULCAN NARVAEZ EDITH MARITZA</t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C25" s="2" t="n">
         <v>19795.02</v>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D25" s="2" t="n">
         <v>2389</v>
       </c>
-      <c r="E24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2" t="n">
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="2" t="n">
         <v>7000</v>
       </c>
     </row>
-    <row r="25">
-      <c r="C25" s="6" t="n">
+    <row r="26">
+      <c r="C26" s="6" t="n">
         <v>59467.53</v>
       </c>
-      <c r="D25" s="6" t="n">
+      <c r="D26" s="6" t="n">
         <v>54049.74</v>
       </c>
-      <c r="E25" s="6" t="n">
+      <c r="E26" s="6" t="n">
         <v>15326.68</v>
       </c>
-      <c r="F25" s="6" t="n">
+      <c r="F26" s="6" t="n">
         <v>10672.57</v>
       </c>
-      <c r="G25" s="6" t="n">
+      <c r="G26" s="6" t="n">
         <v>49000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-03-19 11:30:22
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1965,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>-67.69</v>
+        <v>-321.11</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>0</v>
@@ -2782,7 +2782,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-67.69</v>
+        <v>-321.11</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>7000</v>
@@ -2799,7 +2799,7 @@
         <v>15326.68</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>10755.68</v>
+        <v>10502.26</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>49000</v>
@@ -2970,13 +2970,13 @@
         <v>240</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>-67.69</v>
+        <v>-321.11</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>307.69</v>
+        <v>561.11</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>-0.2820416666666666</v>
+        <v>-1.337958333333333</v>
       </c>
     </row>
     <row r="7">
@@ -3181,13 +3181,13 @@
         <v>57256.2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10755.68</v>
+        <v>10502.26</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>46500.52</v>
+        <v>46753.94</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.187851795962708</v>
+        <v>0.1834257250743151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-19 17:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1236,7 +1236,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>150.8</v>
+        <v>472.57</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -2458,7 +2458,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>150.8</v>
+        <v>546.86</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>0</v>
@@ -2799,7 +2799,7 @@
         <v>15326.68</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>10502.26</v>
+        <v>10898.32</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>49000</v>
@@ -2824,7 +2824,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2922,13 +2922,13 @@
         <v>199.5</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>199.5</v>
+        <v>125.21</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>0.3723809523809524</v>
       </c>
     </row>
     <row r="5">
@@ -3138,13 +3138,13 @@
         <v>52623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5234.08</v>
+        <v>5555.85</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>47388.92</v>
+        <v>47067.15</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.09946373258841192</v>
+        <v>0.1055783592725614</v>
       </c>
     </row>
     <row r="14">
@@ -3181,13 +3181,13 @@
         <v>57256.2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10502.26</v>
+        <v>10898.32</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>46753.94</v>
+        <v>46357.88</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1834257250743151</v>
+        <v>0.1903430545512975</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-03-26 13:30:22
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1980,7 +1980,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0</v>
+        <v>10141.34</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>4 de 24</t>
+          <t>5 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2782,7 +2782,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-321.11</v>
+        <v>9820.23</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>7000</v>
@@ -2799,7 +2799,7 @@
         <v>15326.68</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>10898.32</v>
+        <v>21039.66</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>49000</v>
@@ -2822,7 +2822,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3138,13 +3138,13 @@
         <v>52623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>5555.85</v>
+        <v>15697.19</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>47067.15</v>
+        <v>36925.81</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.1055783592725614</v>
+        <v>0.298295232122836</v>
       </c>
     </row>
     <row r="14">
@@ -3181,13 +3181,13 @@
         <v>57256.2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>10898.32</v>
+        <v>21039.66</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>46357.88</v>
+        <v>36216.54</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1903430545512975</v>
+        <v>0.3674651828098965</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-10 16:15:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1800,7 +1800,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="2" t="n">
-        <v>0</v>
+        <v>740.59</v>
       </c>
       <c r="N22" s="2" t="n">
         <v>0</v>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2099,7 +2099,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>740.59</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>0</v>
@@ -2799,7 +2799,7 @@
         <v>85825.07000000001</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>0</v>
+        <v>740.59</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>49000</v>
@@ -2822,9 +2822,9 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3114,13 +3114,13 @@
         <v>30950</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>740.59</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>30950</v>
+        <v>30209.41</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>0.02392859450726979</v>
       </c>
     </row>
     <row r="13">
@@ -3181,13 +3181,13 @@
         <v>38331.67000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>740.59</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>38331.67000000001</v>
+        <v>37591.08</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>0.0193205774754922</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-13 08:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -897,7 +897,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>0</v>
+        <v>380.13</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>0</v>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
@@ -2296,7 +2296,7 @@
         <v>5824.86</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>0</v>
+        <v>380.13</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -2799,7 +2799,7 @@
         <v>85825.07000000001</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>740.59</v>
+        <v>1120.72</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>49000</v>
@@ -3090,13 +3090,13 @@
         <v>3250</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>380.13</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3250</v>
+        <v>2869.87</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.1169630769230769</v>
       </c>
     </row>
     <row r="12">
@@ -3181,13 +3181,13 @@
         <v>38331.67000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>740.59</v>
+        <v>1120.72</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37591.08</v>
+        <v>37210.95</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.0193205774754922</v>
+        <v>0.02923744256381211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-04-17 14:30:23
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>3231.36</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>1 de 24</t>
+          <t>2 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2350,7 +2350,7 @@
         <v>6156.27</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>3231.36</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>5000</v>
@@ -2799,7 +2799,7 @@
         <v>85825.07000000001</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>910.8099999999999</v>
+        <v>4142.17</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>49000</v>
@@ -2822,7 +2822,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3114,13 +3114,13 @@
         <v>30950</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>572.33</v>
+        <v>3803.69</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>30377.67</v>
+        <v>27146.31</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.01849208400646204</v>
+        <v>0.1228978998384491</v>
       </c>
     </row>
     <row r="13">
@@ -3181,13 +3181,13 @@
         <v>38331.67000000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>910.8100000000001</v>
+        <v>4142.17</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>37420.86</v>
+        <v>34189.5</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.02376129190301388</v>
+        <v>0.1080612976163052</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-14 10:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1320,7 +1320,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>5801.69</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -1593,7 +1593,7 @@
         <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>0</v>
+        <v>1049.93</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -1620,10 +1620,10 @@
         <v>0</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>3027.2</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0</v>
+        <v>208.24</v>
       </c>
       <c r="O19" s="2" t="n">
         <v>0</v>
@@ -2126,57 +2126,57 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
+          <t>1 de 26</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="L28" s="4" t="inlineStr">
         <is>
           <t>0 de 26</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>0 de 26</t>
+          <t>2 de 26</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>0 de 26</t>
+          <t>1 de 26</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
@@ -2219,7 +2219,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2740,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>5801.69</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -2956,7 +2956,7 @@
         <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>4285.37</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>6500</v>
@@ -3243,7 +3243,7 @@
         <v>6499.16</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>0</v>
+        <v>10087.06</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>49000</v>

</xml_diff>

<commit_message>
Actualización automática 2026-05-19 17:30:21
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1500,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>6757.39</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>2349.95</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>2 de 26</t>
+          <t>4 de 26</t>
         </is>
       </c>
       <c r="N28" s="4" t="inlineStr">
@@ -2875,7 +2875,7 @@
         <v>2356.99</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0</v>
+        <v>6757.39</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>6500</v>
@@ -3037,7 +3037,7 @@
         <v>0</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>42.13</v>
+        <v>2392.08</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>1500</v>
@@ -3243,7 +3243,7 @@
         <v>6499.16</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>10820.34</v>
+        <v>19927.68</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>49000</v>
@@ -3266,7 +3266,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3558,13 +3558,13 @@
         <v>53908</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>9473.33</v>
+        <v>18580.67</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>44434.67</v>
+        <v>35327.33</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.1757314313274468</v>
+        <v>0.344673703346442</v>
       </c>
     </row>
     <row r="13">
@@ -3601,13 +3601,13 @@
         <v>58795.5</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>10820.34</v>
+        <v>19927.68</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>47975.16</v>
+        <v>38867.82</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1840334719493839</v>
+        <v>0.3389320611271271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-05-27 10:30:30
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1320,7 +1320,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="2" t="n">
-        <v>6446.13</v>
+        <v>8179.9</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
@@ -2740,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>6446.13</v>
+        <v>8179.9</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -3243,7 +3243,7 @@
         <v>6499.16</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>20030.27</v>
+        <v>21764.04</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>49000</v>
@@ -3558,13 +3558,13 @@
         <v>53908</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>18580.67</v>
+        <v>20314.44</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>35327.33</v>
+        <v>33593.56</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.344673703346442</v>
+        <v>0.3768353491133041</v>
       </c>
     </row>
     <row r="13">
@@ -3601,13 +3601,13 @@
         <v>58795.5</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>20030.27</v>
+        <v>21764.04</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>38765.23</v>
+        <v>37031.46</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3406769225535968</v>
+        <v>0.3701650636528306</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-08 08:30:22
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IMPORTADORA VEGA S.A.</t>
+          <t>JARAMILLO CARVAJAL NICOLAS ESTEBAN</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JARAMILLO CARVAJAL NICOLAS ESTEBAN</t>
+          <t>MARIN DELGADO BRENDA MARIA</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MARIN DELGADO BRENDA MARIA</t>
+          <t>MATERIALES DE CONSTRUCCION SUPERMACONSVI S.A.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MATERIALES DE CONSTRUCCION SUPERMACONSVI S.A.</t>
+          <t>MEGAMAFERS S.A.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MEGAMAFERS S.A.</t>
+          <t>MORILLO CORRAL RUBI KATERINE</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MORILLO CORRAL RUBI KATERINE</t>
+          <t>MUÑOZ LOZA ROMMEL SEBASTIAN</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MUÑOZ LOZA ROMMEL SEBASTIAN</t>
+          <t>ORTEGA PAREDES RUDHT ELENA</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ORTEGA PAREDES RUDHT ELENA</t>
+          <t>OÑATE PEREZ MERCY YOLANDA</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1680,7 +1680,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>6.69</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>OÑATE PEREZ MERCY YOLANDA</t>
+          <t>PADILLA MIER BERTHA MARIETA</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>6.69</v>
+        <v>0</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PADILLA MIER BERTHA MARIETA</t>
+          <t>PAVIMARSA S.A.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PAVIMARSA S.A.</t>
+          <t>SARZOSA UNDA JOSE DOMINGO</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SARZOSA UNDA JOSE DOMINGO</t>
+          <t>SIGCHOS MORA FRANKLIN PORFIRIO</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SIGCHOS MORA FRANKLIN PORFIRIO</t>
+          <t>TRUJILLO TORRES VINICIO RUBEN</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TRUJILLO TORRES VINICIO RUBEN</t>
+          <t>TULCAN NARVAEZ EDITH MARITZA</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2059,144 +2059,84 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>HIDALGO HIDALGO PEDRO GUSTAVO</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>TULCAN NARVAEZ EDITH MARITZA</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
-        <is>
-          <t>1 de 26</t>
-        </is>
-      </c>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="O28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="P28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="Q28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
-        </is>
-      </c>
-      <c r="R28" s="4" t="inlineStr">
-        <is>
-          <t>0 de 26</t>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="inlineStr">
+        <is>
+          <t>1 de 25</t>
+        </is>
+      </c>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="O27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="R27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-06-12 13:30:31
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>6.32</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>2 de 25</t>
+          <t>4 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2680,7 +2680,7 @@
         <v>10650.37</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46.47</v>
+        <v>52.79</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -2815,7 +2815,7 @@
         <v>6938.84</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-181.45</v>
+        <v>-175.13</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>6500</v>
@@ -3183,7 +3183,7 @@
         <v>58243.44</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>69.16000000000003</v>
+        <v>81.80000000000001</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>49000</v>
@@ -3474,13 +3474,13 @@
         <v>43400</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>248.24</v>
+        <v>260.88</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>43151.76</v>
+        <v>43139.12</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.005719815668202765</v>
+        <v>0.006011059907834101</v>
       </c>
     </row>
     <row r="12">
@@ -3517,13 +3517,13 @@
         <v>48433.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>69.16000000000003</v>
+        <v>81.80000000000001</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>48364.34</v>
+        <v>48351.7</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.001427937274820115</v>
+        <v>0.001688913665128475</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-24 15:30:20
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>6.32</v>
+        <v>38.54</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -2815,7 +2815,7 @@
         <v>6938.84</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>-175.13</v>
+        <v>-142.91</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>5000</v>
@@ -3183,7 +3183,7 @@
         <v>58243.44</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>81.80000000000001</v>
+        <v>114.02</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>48500</v>
@@ -3474,13 +3474,13 @@
         <v>43400</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>260.88</v>
+        <v>293.1</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>43139.12</v>
+        <v>43106.9</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.006011059907834101</v>
+        <v>0.006753456221198158</v>
       </c>
     </row>
     <row r="12">
@@ -3517,13 +3517,13 @@
         <v>48433.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>81.80000000000001</v>
+        <v>114.02</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>48351.7</v>
+        <v>48319.48</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.001688913665128475</v>
+        <v>0.002354155698018934</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-06-26 16:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1680,7 +1680,7 @@
         <v>0</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>6.69</v>
+        <v>323.61</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
@@ -2734,7 +2734,7 @@
         <v>2392.08</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>6.69</v>
+        <v>334.04</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1500</v>
@@ -2913,7 +2913,7 @@
         <v>58243.44</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>348.81</v>
+        <v>676.1600000000001</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -2938,7 +2938,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3132,10 +3132,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>10.43</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0</v>
+        <v>-10.43</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -3204,13 +3204,13 @@
         <v>43400</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>308.58</v>
+        <v>625.5</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>43091.42</v>
+        <v>42774.5</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0.007110138248847926</v>
+        <v>0.01441244239631336</v>
       </c>
     </row>
     <row r="12">
@@ -3247,13 +3247,13 @@
         <v>48433.5</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>348.81</v>
+        <v>676.16</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>48084.69</v>
+        <v>47757.34</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.007201833441729382</v>
+        <v>0.01396058513219156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-17 17:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1533,7 +1533,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1079.91</v>
+        <v>0</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>2 de 25</t>
+          <t>1 de 25</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -2680,7 +2680,7 @@
         <v>7791.96</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>1079.91</v>
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -2913,7 +2913,7 @@
         <v>11843.32</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>12403.64</v>
+        <v>11323.73</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3012,13 +3012,13 @@
         <v>2183</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4319.63</v>
+        <v>3239.72</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-2136.63</v>
+        <v>-1056.72</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.978758589097572</v>
+        <v>1.484067796610169</v>
       </c>
     </row>
     <row r="4">
@@ -3271,13 +3271,13 @@
         <v>35016.2</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>12403.64</v>
+        <v>11323.73</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>22612.56</v>
+        <v>23692.47</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3542257583632718</v>
+        <v>0.3233854615863514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-29 08:30:17
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>2162.71</v>
+        <v>2185.77</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2162.71</v>
+        <v>2185.77</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>4000</v>
@@ -2913,7 +2913,7 @@
         <v>11843.32</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>6888.650000000001</v>
+        <v>6911.71</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -2938,7 +2938,7 @@
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3228,13 +3228,13 @@
         <v>30623</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2039.06</v>
+        <v>2062.12</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>28583.94</v>
+        <v>28560.88</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.06658589948731346</v>
+        <v>0.0673389282565392</v>
       </c>
     </row>
     <row r="13">
@@ -3271,13 +3271,13 @@
         <v>35016.2</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6888.65</v>
+        <v>6911.71</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>28127.55</v>
+        <v>28104.49</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1967275146931991</v>
+        <v>0.1973860670204077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-29 16:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>8450.43</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>2358.59</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1533,7 +1533,7 @@
         <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>1004.02</v>
+        <v>2083.93</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -1560,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>3534.56</v>
+        <v>6198.05</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>6 de 25</t>
+          <t>8 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2356,7 +2356,7 @@
         <v>-37.78</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>3239.72</v>
+        <v>11690.15</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -2518,7 +2518,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>605.85</v>
+        <v>2964.44</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>1000</v>
@@ -2680,7 +2680,7 @@
         <v>7791.96</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>4538.58</v>
+        <v>8281.98</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -2913,7 +2913,7 @@
         <v>11843.32</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>6911.71</v>
+        <v>21464.13</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -2936,7 +2936,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3012,13 +3012,13 @@
         <v>2183</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4243.74</v>
+        <v>5323.65</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-2060.74</v>
+        <v>-3140.65</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>1.943994502977554</v>
+        <v>2.438685295464956</v>
       </c>
     </row>
     <row r="4">
@@ -3228,13 +3228,13 @@
         <v>30623</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2062.12</v>
+        <v>15534.63</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>28560.88</v>
+        <v>15088.37</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.0673389282565392</v>
+        <v>0.5072863533945073</v>
       </c>
     </row>
     <row r="13">
@@ -3271,13 +3271,13 @@
         <v>35016.2</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>6911.71</v>
+        <v>21464.13</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>28104.49</v>
+        <v>13552.07</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.1973860670204077</v>
+        <v>0.6129771362969139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-07-30 16:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>2185.77</v>
+        <v>3902.2</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1980,7 +1980,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0</v>
+        <v>6488.12</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>8 de 25</t>
+          <t>9 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2302,7 +2302,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2185.77</v>
+        <v>3902.2</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>4000</v>
@@ -2869,7 +2869,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>6488.12</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3500</v>
@@ -2913,7 +2913,7 @@
         <v>11843.32</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>21464.13</v>
+        <v>29668.68</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3228,13 +3228,13 @@
         <v>30623</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>15534.63</v>
+        <v>23739.18</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>15088.37</v>
+        <v>6883.82</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.5072863533945073</v>
+        <v>0.7752075237566535</v>
       </c>
     </row>
     <row r="13">
@@ -3271,13 +3271,13 @@
         <v>35016.2</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>21464.13</v>
+        <v>29668.68</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>13552.07</v>
+        <v>5347.52</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6129771362969139</v>
+        <v>0.8472843997920961</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-07 11:30:16
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>0</v>
+        <v>1464.57</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>2 de 25</t>
+          <t>3 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2653,7 +2653,7 @@
         <v>4755.17</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>0</v>
+        <v>1464.57</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>5000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>5749.32</v>
+        <v>7213.889999999999</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-08-17 16:30:17
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1560,7 +1560,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>0</v>
+        <v>28.12</v>
       </c>
       <c r="N18" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>3 de 25</t>
+          <t>4 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2680,7 +2680,7 @@
         <v>8281.98</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>0</v>
+        <v>28.12</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>7213.889999999999</v>
+        <v>7242.01</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3252,13 +3252,13 @@
         <v>32623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6563.93</v>
+        <v>6592.05</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>26059.07</v>
+        <v>26030.95</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.20120559114735</v>
+        <v>0.2020675596971462</v>
       </c>
     </row>
     <row r="14">
@@ -3295,13 +3295,13 @@
         <v>43931.88</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>7213.89</v>
+        <v>7242.01</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>36717.99000000001</v>
+        <v>36689.87</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.164206266610944</v>
+        <v>0.1648463484831516</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-19 17:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>12131.73</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>4 de 25</t>
+          <t>5 de 25</t>
         </is>
       </c>
       <c r="N27" s="4" t="inlineStr">
@@ -2159,7 +2159,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -2761,7 +2761,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>12131.73</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>5000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>7242.01</v>
+        <v>19373.74</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -2936,7 +2936,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3252,13 +3252,13 @@
         <v>32623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>6592.05</v>
+        <v>18723.78</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>26030.95</v>
+        <v>13899.22</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.2020675596971462</v>
+        <v>0.57394414983294</v>
       </c>
     </row>
     <row r="14">
@@ -3295,13 +3295,13 @@
         <v>43931.88</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>7242.01</v>
+        <v>19373.74</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>36689.87</v>
+        <v>24558.14</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.1648463484831516</v>
+        <v>0.4409950131886001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-20 15:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>3293.72</v>
+        <v>5180.61</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2572,7 +2572,7 @@
         <v>1133.57</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>3943.68</v>
+        <v>5830.57</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>5000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>19373.74</v>
+        <v>21260.63</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3252,13 +3252,13 @@
         <v>32623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>18723.78</v>
+        <v>20610.67</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>13899.22</v>
+        <v>12012.33</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.57394414983294</v>
+        <v>0.6317834043466266</v>
       </c>
     </row>
     <row r="14">
@@ -3295,13 +3295,13 @@
         <v>43931.88</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>19373.74</v>
+        <v>21260.63</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>24558.14</v>
+        <v>22671.25</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4409950131886001</v>
+        <v>0.4839453717892336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-20 16:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1440,7 +1440,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1464.57</v>
+        <v>2495.09</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -2653,7 +2653,7 @@
         <v>4755.17</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1464.57</v>
+        <v>2495.09</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>5000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>21260.63</v>
+        <v>22291.15</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3252,13 +3252,13 @@
         <v>32623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20610.67</v>
+        <v>21641.19</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>12012.33</v>
+        <v>10981.81</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.6317834043466266</v>
+        <v>0.6633721607454863</v>
       </c>
     </row>
     <row r="14">
@@ -3295,13 +3295,13 @@
         <v>43931.88</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>21260.63</v>
+        <v>22291.15</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>22671.25</v>
+        <v>21640.73</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.4839453717892336</v>
+        <v>0.50740259692961</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-21 08:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -780,7 +780,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1805.64</v>
+        <v>3673.74</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>5180.61</v>
+        <v>5956.77</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>3902.2</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>1805.64</v>
+        <v>3673.74</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>4000</v>
@@ -2572,7 +2572,7 @@
         <v>1133.57</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>5830.57</v>
+        <v>6606.73</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>5000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>22291.15</v>
+        <v>24935.41</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3252,13 +3252,13 @@
         <v>32623</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>21641.19</v>
+        <v>24285.45</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>10981.81</v>
+        <v>8337.549999999999</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0.6633721607454863</v>
+        <v>0.7444272445820433</v>
       </c>
     </row>
     <row r="14">
@@ -3295,13 +3295,13 @@
         <v>43931.88</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>22291.15</v>
+        <v>24935.41</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>21640.73</v>
+        <v>18996.47</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.50740259692961</v>
+        <v>0.5675926001800969</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-26 16:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0</v>
+        <v>313.06</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>0</v>
@@ -777,7 +777,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>860.8099999999999</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>3673.74</v>
@@ -2066,47 +2066,47 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
+          <t>2 de 25</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>0 de 25</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
           <t>1 de 25</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>0 de 25</t>
         </is>
       </c>
       <c r="M27" s="4" t="inlineStr">
@@ -2302,7 +2302,7 @@
         <v>3902.2</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>3673.74</v>
+        <v>4847.61</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>4000</v>
@@ -2913,7 +2913,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>24868.39</v>
+        <v>26042.26</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3012,13 +3012,13 @@
         <v>2183</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>649.96</v>
+        <v>963.02</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1533.04</v>
+        <v>1219.98</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0.2977370590929913</v>
+        <v>0.4411452130096198</v>
       </c>
     </row>
     <row r="4">
@@ -3228,13 +3228,13 @@
         <v>1467</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>860.8099999999999</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1467</v>
+        <v>606.1900000000001</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>0.5867825494205862</v>
       </c>
     </row>
     <row r="13">
@@ -3295,13 +3295,13 @@
         <v>43931.88</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>24868.39</v>
+        <v>26042.26</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>19063.49</v>
+        <v>17889.62</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.5660670565429933</v>
+        <v>0.5927872879558078</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-08-28 17:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -894,13 +894,13 @@
         <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>409.46</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>51.92</v>
+        <v>2720.64</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1020,7 +1020,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>2393.76</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1500,7 +1500,7 @@
         <v>677.21</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>28.12</v>
+        <v>2595.75</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>6 de 24</t>
+          <t>7 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2296,7 +2296,7 @@
         <v>11690.15</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>51.92</v>
+        <v>3130.1</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>5000</v>
@@ -2377,7 +2377,7 @@
         <v>3502.7</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>2393.76</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>3000</v>
@@ -2620,7 +2620,7 @@
         <v>8281.98</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>705.33</v>
+        <v>3272.96</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>6000</v>
@@ -2853,7 +2853,7 @@
         <v>46941.5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>26719.47</v>
+        <v>34759.04</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>48500</v>
@@ -3096,13 +3096,13 @@
         <v>407</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>0</v>
+        <v>409.46</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>407</v>
+        <v>-2.45999999999998</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>0</v>
+        <v>1.006044226044226</v>
       </c>
     </row>
     <row r="10">
@@ -3168,13 +3168,13 @@
         <v>32623</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>24337.37</v>
+        <v>31967.48</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>8285.630000000001</v>
+        <v>655.5200000000004</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0.7460187597707139</v>
+        <v>0.9799062011464305</v>
       </c>
     </row>
     <row r="13">
@@ -3211,13 +3211,13 @@
         <v>38741.88</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>26719.47</v>
+        <v>34759.04</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>12022.41</v>
+        <v>3982.840000000001</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6896792308478575</v>
+        <v>0.897195489738753</v>
       </c>
     </row>
   </sheetData>

</xml_diff>